<commit_message>
Enhance shift handling in attendance application by introducing shiftLabel function for better shift code representation. Update components to utilize new shift labels, improving clarity in shift selection and display. Refactor related logic in calc and excel modules for consistency in shift management.
</commit_message>
<xml_diff>
--- a/public/templates/attendance_template.xlsx
+++ b/public/templates/attendance_template.xlsx
@@ -57,7 +57,7 @@
     <t>20日</t>
   </si>
   <si>
-    <t>○＝終日、△＝半日（0.5日）。有休の午前半休は3.5時間、午後半休は4.0時間。B-2は09:00–18:00（休憩1時間、実働8.0h、午前3.5h・午後4.5h）。Dは08:30–12:30（実働4.0h）。超え勤務は所定の始業前・終業後に在籍した分。</t>
+    <t>○＝終日、△＝半日（0.5日）。有休の午前半休は3.5時間、午後半休は4.0時間。日勤 (8H) は09:00–18:00（休憩1時間、実働8.0h）。半日 (4H) は08:30–12:30（実働4.0h）。所定が8時間の日は日勤、4時間の日は半日の列に印を付けます。超え勤務は所定の始業前・終業後に在籍した分。</t>
   </si>
   <si>
     <t>曜</t>
@@ -66,7 +66,7 @@
     <t>休暇・区分</t>
   </si>
   <si>
-    <t>勤務記号</t>
+    <t>勤務</t>
   </si>
   <si>
     <t>時間外・休日</t>
@@ -90,12 +90,12 @@
     <t>有休</t>
   </si>
   <si>
-    <t xml:space="preserve">B-2
+    <t xml:space="preserve">日勤
 (8H)</t>
   </si>
   <si>
-    <t xml:space="preserve">D
-(4H木土)</t>
+    <t xml:space="preserve">半日
+(4H)</t>
   </si>
   <si>
     <t>始業</t>
@@ -140,14 +140,15 @@
     <t>リハビリフルタイムパート</t>
   </si>
   <si>
-    <t>○＝終日、△＝半日（0.5日）。有休の午前半休は3.5時間、午後半休は4.0時間。A-1は08:30–17:30（休憩1時間、実働8.0h、午前3.5h・午後4.5h）。Dは08:30–12:30（実働4.0h）。7.5Hは08:30–17:00（休憩1時間、実働7.5h、午前3.5h・午後4.0h）。超え勤務は所定の始業前・終業後に在籍した分。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A-1
+    <t>○＝終日、△＝半日（0.5日）。有休の午前半休は3.5時間、午後半休は4.0時間。フル (8H) は08:30–17:30（休憩1時間、実働8.0h）。日勤 (7.5H) は08:30–17:00（休憩1時間、実働7.5h）。半日 (4H) は08:30–12:30（実働4.0h）。所定時間に合う列へ印を付けます。超え勤務は所定の始業前・終業後に在籍した分。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">フル
 (8H)</t>
   </si>
   <si>
-    <t>7.5H</t>
+    <t xml:space="preserve">日勤
+(7.5H)</t>
   </si>
 </sst>
 </file>
@@ -805,8 +806,7 @@
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
     <col min="3" max="6" width="7" customWidth="1"/>
-    <col min="7" max="8" width="11" customWidth="1"/>
-    <col min="9" max="10" width="12" customWidth="1"/>
+    <col min="7" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
     <col min="13" max="13" width="28" customWidth="1"/>
@@ -1640,8 +1640,7 @@
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
     <col min="3" max="6" width="7" customWidth="1"/>
-    <col min="7" max="9" width="11" customWidth="1"/>
-    <col min="10" max="11" width="12" customWidth="1"/>
+    <col min="7" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
     <col min="14" max="14" width="28" customWidth="1"/>

</xml_diff>

<commit_message>
Enhance attendance export functionality by introducing hours context management. Update the renderAttendance function to accept hours context for improved attendance calculations. Refactor related components to support new contract hours and half-day rules, enhancing overall attendance summary accuracy and user experience.
</commit_message>
<xml_diff>
--- a/public/templates/attendance_template.xlsx
+++ b/public/templates/attendance_template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="46">
   <si>
     <t>出勤簿</t>
   </si>
@@ -135,6 +135,15 @@
   </si>
   <si>
     <t>半日未満（回）</t>
+  </si>
+  <si>
+    <t>勤務時間合計</t>
+  </si>
+  <si>
+    <t>有休時間合計</t>
+  </si>
+  <si>
+    <t>支給対象時間</t>
   </si>
   <si>
     <t>リハビリフルタイムパート</t>
@@ -800,7 +809,7 @@
     <tabColor rgb="FF0F5C61"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1581,24 +1590,75 @@
       <c r="M47" s="19"/>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
+      <c r="A48" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
-      <c r="H48" s="21"/>
-      <c r="I48" s="21"/>
-      <c r="J48" s="21"/>
-      <c r="K48" s="21"/>
-      <c r="L48" s="21"/>
-      <c r="M48" s="22"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="19"/>
+    </row>
+    <row r="49" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A49" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B49" s="17"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="18"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="19"/>
+    </row>
+    <row r="50" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" s="17"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="19"/>
+    </row>
+    <row r="51" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A51" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B51" s="20"/>
+      <c r="C51" s="21"/>
+      <c r="D51" s="21"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="21"/>
+      <c r="G51" s="21"/>
+      <c r="H51" s="21"/>
+      <c r="I51" s="21"/>
+      <c r="J51" s="21"/>
+      <c r="K51" s="21"/>
+      <c r="L51" s="21"/>
+      <c r="M51" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="22">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
@@ -1618,6 +1678,9 @@
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
@@ -1634,7 +1697,7 @@
     <tabColor rgb="FF0F5C61"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1685,7 +1748,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1738,7 +1801,7 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -1800,13 +1863,13 @@
         <v>23</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>25</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>26</v>
@@ -2463,25 +2526,79 @@
       <c r="N47" s="19"/>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
+      <c r="A48" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
-      <c r="H48" s="21"/>
-      <c r="I48" s="21"/>
-      <c r="J48" s="21"/>
-      <c r="K48" s="21"/>
-      <c r="L48" s="21"/>
-      <c r="M48" s="21"/>
-      <c r="N48" s="22"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="18"/>
+      <c r="N48" s="19"/>
+    </row>
+    <row r="49" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B49" s="17"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="18"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18"/>
+      <c r="N49" s="19"/>
+    </row>
+    <row r="50" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" s="17"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18"/>
+      <c r="N50" s="19"/>
+    </row>
+    <row r="51" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B51" s="20"/>
+      <c r="C51" s="21"/>
+      <c r="D51" s="21"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="21"/>
+      <c r="G51" s="21"/>
+      <c r="H51" s="21"/>
+      <c r="I51" s="21"/>
+      <c r="J51" s="21"/>
+      <c r="K51" s="21"/>
+      <c r="L51" s="21"/>
+      <c r="M51" s="21"/>
+      <c r="N51" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="22">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
@@ -2501,6 +2618,9 @@
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Refactor attendance file naming and improve Excel export functionality. Update attendance file name format to include year and month directly, enhancing clarity. Refactor writeAttendance function to ensure proper handling of cell values without altering formatting, and introduce footer writing logic for better summary presentation. Adjust page setup properties in template creation for consistent printing layout.
</commit_message>
<xml_diff>
--- a/public/templates/attendance_template.xlsx
+++ b/public/templates/attendance_template.xlsx
@@ -1684,7 +1684,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup paperSize="8" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <headerFooter>
     <oddFooter>&amp;L勤怠クラフト&amp;C&amp;A&amp;R&amp;P / &amp;N</oddFooter>
   </headerFooter>
@@ -2624,7 +2624,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup paperSize="8" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <headerFooter>
     <oddFooter>&amp;L勤怠クラフト&amp;C&amp;A&amp;R&amp;P / &amp;N</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Refactor time formatting and Excel export logic for attendance. Update time display to include hours and minutes in the format "X時間YY分 (X.Xh)". Introduce new summary label for paid leave hours. Refactor Excel writing functions to ensure proper handling of merged cells and improve footer presentation. Enhance alignment settings in the template for better readability.
</commit_message>
<xml_diff>
--- a/public/templates/attendance_template.xlsx
+++ b/public/templates/attendance_template.xlsx
@@ -251,7 +251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -335,21 +335,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF9AA5A6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF1F2937"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF9AA5A6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF9AA5A6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF1F2937"/>
       </left>
@@ -379,26 +364,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF9AA5A6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF1F2937"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF9AA5A6"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF1F2937"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -443,28 +413,22 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1485,7 +1449,7 @@
       <c r="J41" s="18"/>
       <c r="K41" s="18"/>
       <c r="L41" s="18"/>
-      <c r="M41" s="19"/>
+      <c r="M41" s="18"/>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
@@ -1502,7 +1466,7 @@
       <c r="J42" s="18"/>
       <c r="K42" s="18"/>
       <c r="L42" s="18"/>
-      <c r="M42" s="19"/>
+      <c r="M42" s="18"/>
     </row>
     <row r="43" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
@@ -1519,7 +1483,7 @@
       <c r="J43" s="18"/>
       <c r="K43" s="18"/>
       <c r="L43" s="18"/>
-      <c r="M43" s="19"/>
+      <c r="M43" s="18"/>
     </row>
     <row r="44" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
@@ -1536,7 +1500,7 @@
       <c r="J44" s="18"/>
       <c r="K44" s="18"/>
       <c r="L44" s="18"/>
-      <c r="M44" s="19"/>
+      <c r="M44" s="18"/>
     </row>
     <row r="45" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
@@ -1553,7 +1517,7 @@
       <c r="J45" s="18"/>
       <c r="K45" s="18"/>
       <c r="L45" s="18"/>
-      <c r="M45" s="19"/>
+      <c r="M45" s="18"/>
     </row>
     <row r="46" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
@@ -1570,7 +1534,7 @@
       <c r="J46" s="18"/>
       <c r="K46" s="18"/>
       <c r="L46" s="18"/>
-      <c r="M46" s="19"/>
+      <c r="M46" s="18"/>
     </row>
     <row r="47" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
@@ -1587,7 +1551,7 @@
       <c r="J47" s="18"/>
       <c r="K47" s="18"/>
       <c r="L47" s="18"/>
-      <c r="M47" s="19"/>
+      <c r="M47" s="18"/>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
@@ -1604,7 +1568,7 @@
       <c r="J48" s="18"/>
       <c r="K48" s="18"/>
       <c r="L48" s="18"/>
-      <c r="M48" s="19"/>
+      <c r="M48" s="18"/>
     </row>
     <row r="49" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
@@ -1621,7 +1585,7 @@
       <c r="J49" s="18"/>
       <c r="K49" s="18"/>
       <c r="L49" s="18"/>
-      <c r="M49" s="19"/>
+      <c r="M49" s="18"/>
     </row>
     <row r="50" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="17" t="s">
@@ -1638,27 +1602,27 @@
       <c r="J50" s="18"/>
       <c r="K50" s="18"/>
       <c r="L50" s="18"/>
-      <c r="M50" s="19"/>
+      <c r="M50" s="18"/>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A51" s="20" t="s">
+      <c r="A51" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B51" s="20"/>
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21"/>
-      <c r="K51" s="21"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="22"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="20"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
+      <c r="L51" s="20"/>
+      <c r="M51" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="33">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
@@ -1671,16 +1635,27 @@
     <mergeCell ref="M6:M7"/>
     <mergeCell ref="A40:B40"/>
     <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:M41"/>
     <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:M42"/>
     <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:M43"/>
     <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:M44"/>
     <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:M45"/>
     <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:M46"/>
     <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:M47"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:M48"/>
     <mergeCell ref="A49:B49"/>
+    <mergeCell ref="C49:M49"/>
     <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C50:M50"/>
     <mergeCell ref="A51:B51"/>
+    <mergeCell ref="C51:M51"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
@@ -2415,7 +2390,7 @@
       <c r="K41" s="18"/>
       <c r="L41" s="18"/>
       <c r="M41" s="18"/>
-      <c r="N41" s="19"/>
+      <c r="N41" s="18"/>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
@@ -2433,7 +2408,7 @@
       <c r="K42" s="18"/>
       <c r="L42" s="18"/>
       <c r="M42" s="18"/>
-      <c r="N42" s="19"/>
+      <c r="N42" s="18"/>
     </row>
     <row r="43" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
@@ -2451,7 +2426,7 @@
       <c r="K43" s="18"/>
       <c r="L43" s="18"/>
       <c r="M43" s="18"/>
-      <c r="N43" s="19"/>
+      <c r="N43" s="18"/>
     </row>
     <row r="44" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
@@ -2469,7 +2444,7 @@
       <c r="K44" s="18"/>
       <c r="L44" s="18"/>
       <c r="M44" s="18"/>
-      <c r="N44" s="19"/>
+      <c r="N44" s="18"/>
     </row>
     <row r="45" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
@@ -2487,7 +2462,7 @@
       <c r="K45" s="18"/>
       <c r="L45" s="18"/>
       <c r="M45" s="18"/>
-      <c r="N45" s="19"/>
+      <c r="N45" s="18"/>
     </row>
     <row r="46" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
@@ -2505,7 +2480,7 @@
       <c r="K46" s="18"/>
       <c r="L46" s="18"/>
       <c r="M46" s="18"/>
-      <c r="N46" s="19"/>
+      <c r="N46" s="18"/>
     </row>
     <row r="47" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
@@ -2523,7 +2498,7 @@
       <c r="K47" s="18"/>
       <c r="L47" s="18"/>
       <c r="M47" s="18"/>
-      <c r="N47" s="19"/>
+      <c r="N47" s="18"/>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
@@ -2541,7 +2516,7 @@
       <c r="K48" s="18"/>
       <c r="L48" s="18"/>
       <c r="M48" s="18"/>
-      <c r="N48" s="19"/>
+      <c r="N48" s="18"/>
     </row>
     <row r="49" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
@@ -2559,7 +2534,7 @@
       <c r="K49" s="18"/>
       <c r="L49" s="18"/>
       <c r="M49" s="18"/>
-      <c r="N49" s="19"/>
+      <c r="N49" s="18"/>
     </row>
     <row r="50" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="17" t="s">
@@ -2577,28 +2552,28 @@
       <c r="K50" s="18"/>
       <c r="L50" s="18"/>
       <c r="M50" s="18"/>
-      <c r="N50" s="19"/>
+      <c r="N50" s="18"/>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A51" s="20" t="s">
+      <c r="A51" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B51" s="20"/>
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21"/>
-      <c r="K51" s="21"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
-      <c r="N51" s="22"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="20"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
+      <c r="L51" s="20"/>
+      <c r="M51" s="20"/>
+      <c r="N51" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="33">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
@@ -2611,16 +2586,27 @@
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="A40:B40"/>
     <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:N41"/>
     <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:N42"/>
     <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:N43"/>
     <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:N44"/>
     <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:N45"/>
     <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:N46"/>
     <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:N47"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:N48"/>
     <mergeCell ref="A49:B49"/>
+    <mergeCell ref="C49:N49"/>
     <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C50:N50"/>
     <mergeCell ref="A51:B51"/>
+    <mergeCell ref="C51:N51"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>

</xml_diff>